<commit_message>
Fixed the no such file found error
</commit_message>
<xml_diff>
--- a/XLSXs/DeRec-GEA20 - 24_refactoring_data.xlsx
+++ b/XLSXs/DeRec-GEA20 - 24_refactoring_data.xlsx
@@ -270,34 +270,34 @@
         <v>0.0</v>
       </c>
       <c r="H2" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="I2" t="n" s="0">
         <v>-1.0</v>
       </c>
       <c r="J2" t="n" s="0">
-        <v>-1.0</v>
+        <v>105.0</v>
       </c>
       <c r="K2" t="n" s="0">
-        <v>-1.0</v>
+        <v>57.0</v>
       </c>
       <c r="L2" t="n" s="0">
-        <v>-1.0</v>
+        <v>15.0</v>
       </c>
       <c r="M2" t="n" s="0">
-        <v>-1.0</v>
+        <v>72.0</v>
       </c>
       <c r="N2" t="n" s="0">
-        <v>-1.0</v>
+        <v>3.0</v>
       </c>
       <c r="O2" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="P2" t="n" s="0">
-        <v>-1.0</v>
+        <v>6.0</v>
       </c>
       <c r="Q2" t="n" s="0">
-        <v>-1.0</v>
+        <v>80.0</v>
       </c>
     </row>
     <row r="3">
@@ -317,34 +317,34 @@
         <v>0.0</v>
       </c>
       <c r="H3" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="I3" t="n" s="0">
         <v>-1.0</v>
       </c>
       <c r="J3" t="n" s="0">
-        <v>-1.0</v>
+        <v>1.0</v>
       </c>
       <c r="K3" t="n" s="0">
-        <v>-1.0</v>
+        <v>11.0</v>
       </c>
       <c r="L3" t="n" s="0">
-        <v>-1.0</v>
+        <v>2.0</v>
       </c>
       <c r="M3" t="n" s="0">
-        <v>-1.0</v>
+        <v>13.0</v>
       </c>
       <c r="N3" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="O3" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="P3" t="n" s="0">
-        <v>-1.0</v>
+        <v>2.0</v>
       </c>
       <c r="Q3" t="n" s="0">
-        <v>-1.0</v>
+        <v>19.0</v>
       </c>
     </row>
     <row r="4">
@@ -364,34 +364,34 @@
         <v>0.0</v>
       </c>
       <c r="H4" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="I4" t="n" s="0">
         <v>-1.0</v>
       </c>
       <c r="J4" t="n" s="0">
-        <v>-1.0</v>
+        <v>28.0</v>
       </c>
       <c r="K4" t="n" s="0">
-        <v>-1.0</v>
+        <v>17.0</v>
       </c>
       <c r="L4" t="n" s="0">
-        <v>-1.0</v>
+        <v>8.0</v>
       </c>
       <c r="M4" t="n" s="0">
-        <v>-1.0</v>
+        <v>25.0</v>
       </c>
       <c r="N4" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="O4" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="P4" t="n" s="0">
-        <v>-1.0</v>
+        <v>3.0</v>
       </c>
       <c r="Q4" t="n" s="0">
-        <v>-1.0</v>
+        <v>70.0</v>
       </c>
     </row>
     <row r="5">
@@ -411,34 +411,34 @@
         <v>0.0</v>
       </c>
       <c r="H5" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="I5" t="n" s="0">
         <v>-1.0</v>
       </c>
       <c r="J5" t="n" s="0">
-        <v>-1.0</v>
+        <v>3.0</v>
       </c>
       <c r="K5" t="n" s="0">
-        <v>-1.0</v>
+        <v>3.0</v>
       </c>
       <c r="L5" t="n" s="0">
-        <v>-1.0</v>
+        <v>3.0</v>
       </c>
       <c r="M5" t="n" s="0">
-        <v>-1.0</v>
+        <v>6.0</v>
       </c>
       <c r="N5" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="O5" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="P5" t="n" s="0">
-        <v>-1.0</v>
+        <v>1.0</v>
       </c>
       <c r="Q5" t="n" s="0">
-        <v>-1.0</v>
+        <v>14.0</v>
       </c>
     </row>
     <row r="6">
@@ -458,34 +458,34 @@
         <v>0.0</v>
       </c>
       <c r="H6" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="I6" t="n" s="0">
         <v>-1.0</v>
       </c>
       <c r="J6" t="n" s="0">
-        <v>-1.0</v>
+        <v>28.0</v>
       </c>
       <c r="K6" t="n" s="0">
-        <v>-1.0</v>
+        <v>19.0</v>
       </c>
       <c r="L6" t="n" s="0">
-        <v>-1.0</v>
+        <v>8.0</v>
       </c>
       <c r="M6" t="n" s="0">
-        <v>-1.0</v>
+        <v>27.0</v>
       </c>
       <c r="N6" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="O6" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="P6" t="n" s="0">
-        <v>-1.0</v>
+        <v>2.0</v>
       </c>
       <c r="Q6" t="n" s="0">
-        <v>-1.0</v>
+        <v>56.0</v>
       </c>
     </row>
     <row r="7">
@@ -505,34 +505,34 @@
         <v>0.0</v>
       </c>
       <c r="H7" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="I7" t="n" s="0">
         <v>-1.0</v>
       </c>
       <c r="J7" t="n" s="0">
-        <v>-1.0</v>
+        <v>120.0</v>
       </c>
       <c r="K7" t="n" s="0">
-        <v>-1.0</v>
+        <v>42.0</v>
       </c>
       <c r="L7" t="n" s="0">
-        <v>-1.0</v>
+        <v>16.0</v>
       </c>
       <c r="M7" t="n" s="0">
-        <v>-1.0</v>
+        <v>58.0</v>
       </c>
       <c r="N7" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="O7" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="P7" t="n" s="0">
-        <v>-1.0</v>
+        <v>2.0</v>
       </c>
       <c r="Q7" t="n" s="0">
-        <v>-1.0</v>
+        <v>134.0</v>
       </c>
     </row>
     <row r="8">
@@ -552,34 +552,34 @@
         <v>0.0</v>
       </c>
       <c r="H8" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="I8" t="n" s="0">
         <v>-1.0</v>
       </c>
       <c r="J8" t="n" s="0">
-        <v>-1.0</v>
+        <v>3.0</v>
       </c>
       <c r="K8" t="n" s="0">
-        <v>-1.0</v>
+        <v>17.0</v>
       </c>
       <c r="L8" t="n" s="0">
-        <v>-1.0</v>
+        <v>3.0</v>
       </c>
       <c r="M8" t="n" s="0">
-        <v>-1.0</v>
+        <v>20.0</v>
       </c>
       <c r="N8" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="O8" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="P8" t="n" s="0">
-        <v>-1.0</v>
+        <v>4.0</v>
       </c>
       <c r="Q8" t="n" s="0">
-        <v>-1.0</v>
+        <v>47.0</v>
       </c>
     </row>
     <row r="9">
@@ -599,34 +599,34 @@
         <v>0.0</v>
       </c>
       <c r="H9" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="I9" t="n" s="0">
         <v>-1.0</v>
       </c>
       <c r="J9" t="n" s="0">
-        <v>-1.0</v>
+        <v>28.0</v>
       </c>
       <c r="K9" t="n" s="0">
-        <v>-1.0</v>
+        <v>31.0</v>
       </c>
       <c r="L9" t="n" s="0">
-        <v>-1.0</v>
+        <v>8.0</v>
       </c>
       <c r="M9" t="n" s="0">
-        <v>-1.0</v>
+        <v>39.0</v>
       </c>
       <c r="N9" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="O9" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="P9" t="n" s="0">
-        <v>-1.0</v>
+        <v>4.0</v>
       </c>
       <c r="Q9" t="n" s="0">
-        <v>-1.0</v>
+        <v>77.0</v>
       </c>
     </row>
     <row r="10">
@@ -646,34 +646,34 @@
         <v>0.0</v>
       </c>
       <c r="H10" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="I10" t="n" s="0">
         <v>-1.0</v>
       </c>
       <c r="J10" t="n" s="0">
-        <v>-1.0</v>
+        <v>6.0</v>
       </c>
       <c r="K10" t="n" s="0">
-        <v>-1.0</v>
+        <v>16.0</v>
       </c>
       <c r="L10" t="n" s="0">
-        <v>-1.0</v>
+        <v>4.0</v>
       </c>
       <c r="M10" t="n" s="0">
-        <v>-1.0</v>
+        <v>20.0</v>
       </c>
       <c r="N10" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="O10" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="P10" t="n" s="0">
-        <v>-1.0</v>
+        <v>1.0</v>
       </c>
       <c r="Q10" t="n" s="0">
-        <v>-1.0</v>
+        <v>37.0</v>
       </c>
     </row>
     <row r="11">
@@ -693,34 +693,34 @@
         <v>0.0</v>
       </c>
       <c r="H11" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="I11" t="n" s="0">
         <v>-1.0</v>
       </c>
       <c r="J11" t="n" s="0">
-        <v>-1.0</v>
+        <v>6.0</v>
       </c>
       <c r="K11" t="n" s="0">
-        <v>-1.0</v>
+        <v>19.0</v>
       </c>
       <c r="L11" t="n" s="0">
-        <v>-1.0</v>
+        <v>4.0</v>
       </c>
       <c r="M11" t="n" s="0">
-        <v>-1.0</v>
+        <v>23.0</v>
       </c>
       <c r="N11" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="O11" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="P11" t="n" s="0">
-        <v>-1.0</v>
+        <v>2.0</v>
       </c>
       <c r="Q11" t="n" s="0">
-        <v>-1.0</v>
+        <v>28.0</v>
       </c>
     </row>
     <row r="12">
@@ -740,34 +740,34 @@
         <v>0.0</v>
       </c>
       <c r="H12" t="n" s="0">
-        <v>-1.0</v>
+        <v>1.0</v>
       </c>
       <c r="I12" t="n" s="0">
         <v>-1.0</v>
       </c>
       <c r="J12" t="n" s="0">
-        <v>-1.0</v>
+        <v>21.0</v>
       </c>
       <c r="K12" t="n" s="0">
-        <v>-1.0</v>
+        <v>10.0</v>
       </c>
       <c r="L12" t="n" s="0">
-        <v>-1.0</v>
+        <v>7.0</v>
       </c>
       <c r="M12" t="n" s="0">
-        <v>-1.0</v>
+        <v>17.0</v>
       </c>
       <c r="N12" t="n" s="0">
-        <v>-1.0</v>
+        <v>1.0</v>
       </c>
       <c r="O12" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="P12" t="n" s="0">
-        <v>-1.0</v>
+        <v>3.0</v>
       </c>
       <c r="Q12" t="n" s="0">
-        <v>-1.0</v>
+        <v>38.0</v>
       </c>
     </row>
     <row r="13">
@@ -787,34 +787,34 @@
         <v>0.0</v>
       </c>
       <c r="H13" t="n" s="0">
-        <v>-1.0</v>
+        <v>1.0</v>
       </c>
       <c r="I13" t="n" s="0">
         <v>-1.0</v>
       </c>
       <c r="J13" t="n" s="0">
-        <v>-1.0</v>
+        <v>1.0</v>
       </c>
       <c r="K13" t="n" s="0">
-        <v>-1.0</v>
+        <v>13.0</v>
       </c>
       <c r="L13" t="n" s="0">
-        <v>-1.0</v>
+        <v>2.0</v>
       </c>
       <c r="M13" t="n" s="0">
-        <v>-1.0</v>
+        <v>15.0</v>
       </c>
       <c r="N13" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="O13" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="P13" t="n" s="0">
-        <v>-1.0</v>
+        <v>3.0</v>
       </c>
       <c r="Q13" t="n" s="0">
-        <v>-1.0</v>
+        <v>24.0</v>
       </c>
     </row>
     <row r="14">
@@ -834,34 +834,34 @@
         <v>0.0</v>
       </c>
       <c r="H14" t="n" s="0">
-        <v>-1.0</v>
+        <v>2.0</v>
       </c>
       <c r="I14" t="n" s="0">
         <v>-1.0</v>
       </c>
       <c r="J14" t="n" s="0">
-        <v>-1.0</v>
+        <v>10.0</v>
       </c>
       <c r="K14" t="n" s="0">
-        <v>-1.0</v>
+        <v>17.0</v>
       </c>
       <c r="L14" t="n" s="0">
-        <v>-1.0</v>
+        <v>5.0</v>
       </c>
       <c r="M14" t="n" s="0">
-        <v>-1.0</v>
+        <v>22.0</v>
       </c>
       <c r="N14" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="O14" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="P14" t="n" s="0">
-        <v>-1.0</v>
+        <v>3.0</v>
       </c>
       <c r="Q14" t="n" s="0">
-        <v>-1.0</v>
+        <v>33.0</v>
       </c>
     </row>
     <row r="15">
@@ -881,34 +881,34 @@
         <v>0.0</v>
       </c>
       <c r="H15" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="I15" t="n" s="0">
         <v>-1.0</v>
       </c>
       <c r="J15" t="n" s="0">
-        <v>-1.0</v>
+        <v>3.0</v>
       </c>
       <c r="K15" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="L15" t="n" s="0">
-        <v>-1.0</v>
+        <v>3.0</v>
       </c>
       <c r="M15" t="n" s="0">
-        <v>-1.0</v>
+        <v>3.0</v>
       </c>
       <c r="N15" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="O15" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="P15" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="Q15" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
     </row>
     <row r="16">
@@ -928,34 +928,34 @@
         <v>0.0</v>
       </c>
       <c r="H16" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="I16" t="n" s="0">
         <v>-1.0</v>
       </c>
       <c r="J16" t="n" s="0">
-        <v>-1.0</v>
+        <v>10.0</v>
       </c>
       <c r="K16" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="L16" t="n" s="0">
-        <v>-1.0</v>
+        <v>5.0</v>
       </c>
       <c r="M16" t="n" s="0">
-        <v>-1.0</v>
+        <v>5.0</v>
       </c>
       <c r="N16" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="O16" t="n" s="0">
-        <v>-1.0</v>
+        <v>3.0</v>
       </c>
       <c r="P16" t="n" s="0">
-        <v>-1.0</v>
+        <v>1.0</v>
       </c>
       <c r="Q16" t="n" s="0">
-        <v>-1.0</v>
+        <v>8.0</v>
       </c>
     </row>
     <row r="17">
@@ -975,34 +975,34 @@
         <v>0.0</v>
       </c>
       <c r="H17" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="I17" t="n" s="0">
         <v>-1.0</v>
       </c>
       <c r="J17" t="n" s="0">
-        <v>-1.0</v>
+        <v>1.0</v>
       </c>
       <c r="K17" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="L17" t="n" s="0">
-        <v>-1.0</v>
+        <v>2.0</v>
       </c>
       <c r="M17" t="n" s="0">
-        <v>-1.0</v>
+        <v>2.0</v>
       </c>
       <c r="N17" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="O17" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="P17" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="Q17" t="n" s="0">
-        <v>-1.0</v>
+        <v>4.0</v>
       </c>
     </row>
     <row r="18">
@@ -1022,34 +1022,34 @@
         <v>0.0</v>
       </c>
       <c r="H18" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="I18" t="n" s="0">
         <v>-1.0</v>
       </c>
       <c r="J18" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="K18" t="n" s="0">
-        <v>-1.0</v>
+        <v>2.0</v>
       </c>
       <c r="L18" t="n" s="0">
-        <v>-1.0</v>
+        <v>1.0</v>
       </c>
       <c r="M18" t="n" s="0">
-        <v>-1.0</v>
+        <v>3.0</v>
       </c>
       <c r="N18" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="O18" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="P18" t="n" s="0">
-        <v>-1.0</v>
+        <v>1.0</v>
       </c>
       <c r="Q18" t="n" s="0">
-        <v>-1.0</v>
+        <v>13.0</v>
       </c>
     </row>
     <row r="19">
@@ -1069,34 +1069,34 @@
         <v>0.0</v>
       </c>
       <c r="H19" t="n" s="0">
-        <v>-1.0</v>
+        <v>1.0</v>
       </c>
       <c r="I19" t="n" s="0">
         <v>-1.0</v>
       </c>
       <c r="J19" t="n" s="0">
-        <v>-1.0</v>
+        <v>276.0</v>
       </c>
       <c r="K19" t="n" s="0">
-        <v>-1.0</v>
+        <v>14.0</v>
       </c>
       <c r="L19" t="n" s="0">
-        <v>-1.0</v>
+        <v>24.0</v>
       </c>
       <c r="M19" t="n" s="0">
-        <v>-1.0</v>
+        <v>38.0</v>
       </c>
       <c r="N19" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="O19" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="P19" t="n" s="0">
-        <v>-1.0</v>
+        <v>2.0</v>
       </c>
       <c r="Q19" t="n" s="0">
-        <v>-1.0</v>
+        <v>146.0</v>
       </c>
     </row>
     <row r="20">
@@ -1116,34 +1116,34 @@
         <v>0.0</v>
       </c>
       <c r="H20" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="I20" t="n" s="0">
         <v>-1.0</v>
       </c>
       <c r="J20" t="n" s="0">
-        <v>-1.0</v>
+        <v>406.0</v>
       </c>
       <c r="K20" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="L20" t="n" s="0">
-        <v>-1.0</v>
+        <v>29.0</v>
       </c>
       <c r="M20" t="n" s="0">
-        <v>-1.0</v>
+        <v>29.0</v>
       </c>
       <c r="N20" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="O20" t="n" s="0">
-        <v>-1.0</v>
+        <v>2.0</v>
       </c>
       <c r="P20" t="n" s="0">
-        <v>-1.0</v>
+        <v>1.0</v>
       </c>
       <c r="Q20" t="n" s="0">
-        <v>-1.0</v>
+        <v>83.0</v>
       </c>
     </row>
     <row r="21">
@@ -1163,34 +1163,34 @@
         <v>0.0</v>
       </c>
       <c r="H21" t="n" s="0">
-        <v>-1.0</v>
+        <v>2.0</v>
       </c>
       <c r="I21" t="n" s="0">
         <v>-1.0</v>
       </c>
       <c r="J21" t="n" s="0">
-        <v>-1.0</v>
+        <v>6.0</v>
       </c>
       <c r="K21" t="n" s="0">
-        <v>-1.0</v>
+        <v>30.0</v>
       </c>
       <c r="L21" t="n" s="0">
-        <v>-1.0</v>
+        <v>4.0</v>
       </c>
       <c r="M21" t="n" s="0">
-        <v>-1.0</v>
+        <v>34.0</v>
       </c>
       <c r="N21" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="O21" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="P21" t="n" s="0">
-        <v>-1.0</v>
+        <v>4.0</v>
       </c>
       <c r="Q21" t="n" s="0">
-        <v>-1.0</v>
+        <v>74.0</v>
       </c>
     </row>
     <row r="22">
@@ -1210,34 +1210,34 @@
         <v>0.0</v>
       </c>
       <c r="H22" t="n" s="0">
-        <v>-1.0</v>
+        <v>2.0</v>
       </c>
       <c r="I22" t="n" s="0">
         <v>-1.0</v>
       </c>
       <c r="J22" t="n" s="0">
-        <v>-1.0</v>
+        <v>3.0</v>
       </c>
       <c r="K22" t="n" s="0">
-        <v>-1.0</v>
+        <v>12.0</v>
       </c>
       <c r="L22" t="n" s="0">
-        <v>-1.0</v>
+        <v>3.0</v>
       </c>
       <c r="M22" t="n" s="0">
-        <v>-1.0</v>
+        <v>15.0</v>
       </c>
       <c r="N22" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="O22" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="P22" t="n" s="0">
-        <v>-1.0</v>
+        <v>3.0</v>
       </c>
       <c r="Q22" t="n" s="0">
-        <v>-1.0</v>
+        <v>45.0</v>
       </c>
     </row>
     <row r="23">
@@ -1257,34 +1257,34 @@
         <v>0.0</v>
       </c>
       <c r="H23" t="n" s="0">
-        <v>-1.0</v>
+        <v>1.0</v>
       </c>
       <c r="I23" t="n" s="0">
         <v>-1.0</v>
       </c>
       <c r="J23" t="n" s="0">
-        <v>-1.0</v>
+        <v>21.0</v>
       </c>
       <c r="K23" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="L23" t="n" s="0">
-        <v>-1.0</v>
+        <v>7.0</v>
       </c>
       <c r="M23" t="n" s="0">
-        <v>-1.0</v>
+        <v>7.0</v>
       </c>
       <c r="N23" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="O23" t="n" s="0">
-        <v>-1.0</v>
+        <v>2.0</v>
       </c>
       <c r="P23" t="n" s="0">
-        <v>-1.0</v>
+        <v>2.0</v>
       </c>
       <c r="Q23" t="n" s="0">
-        <v>-1.0</v>
+        <v>20.0</v>
       </c>
     </row>
     <row r="24">
@@ -1304,34 +1304,34 @@
         <v>0.0</v>
       </c>
       <c r="H24" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="I24" t="n" s="0">
         <v>-1.0</v>
       </c>
       <c r="J24" t="n" s="0">
-        <v>-1.0</v>
+        <v>1.0</v>
       </c>
       <c r="K24" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="L24" t="n" s="0">
-        <v>-1.0</v>
+        <v>2.0</v>
       </c>
       <c r="M24" t="n" s="0">
-        <v>-1.0</v>
+        <v>2.0</v>
       </c>
       <c r="N24" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="O24" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="P24" t="n" s="0">
-        <v>-1.0</v>
+        <v>2.0</v>
       </c>
       <c r="Q24" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
     </row>
     <row r="25">
@@ -1351,34 +1351,34 @@
         <v>0.0</v>
       </c>
       <c r="H25" t="n" s="0">
-        <v>-1.0</v>
+        <v>1.0</v>
       </c>
       <c r="I25" t="n" s="0">
         <v>-1.0</v>
       </c>
       <c r="J25" t="n" s="0">
-        <v>-1.0</v>
+        <v>10.0</v>
       </c>
       <c r="K25" t="n" s="0">
-        <v>-1.0</v>
+        <v>16.0</v>
       </c>
       <c r="L25" t="n" s="0">
-        <v>-1.0</v>
+        <v>5.0</v>
       </c>
       <c r="M25" t="n" s="0">
-        <v>-1.0</v>
+        <v>21.0</v>
       </c>
       <c r="N25" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="O25" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="P25" t="n" s="0">
-        <v>-1.0</v>
+        <v>3.0</v>
       </c>
       <c r="Q25" t="n" s="0">
-        <v>-1.0</v>
+        <v>47.0</v>
       </c>
     </row>
     <row r="26">
@@ -1398,34 +1398,34 @@
         <v>0.0</v>
       </c>
       <c r="H26" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="I26" t="n" s="0">
         <v>-1.0</v>
       </c>
       <c r="J26" t="n" s="0">
-        <v>-1.0</v>
+        <v>861.0</v>
       </c>
       <c r="K26" t="n" s="0">
-        <v>-1.0</v>
+        <v>205.0</v>
       </c>
       <c r="L26" t="n" s="0">
-        <v>-1.0</v>
+        <v>42.0</v>
       </c>
       <c r="M26" t="n" s="0">
-        <v>-1.0</v>
+        <v>247.0</v>
       </c>
       <c r="N26" t="n" s="0">
-        <v>-1.0</v>
+        <v>2.0</v>
       </c>
       <c r="O26" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="P26" t="n" s="0">
-        <v>-1.0</v>
+        <v>4.0</v>
       </c>
       <c r="Q26" t="n" s="0">
-        <v>-1.0</v>
+        <v>606.0</v>
       </c>
     </row>
     <row r="27">
@@ -1445,34 +1445,34 @@
         <v>0.0</v>
       </c>
       <c r="H27" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="I27" t="n" s="0">
         <v>-1.0</v>
       </c>
       <c r="J27" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="K27" t="n" s="0">
-        <v>-1.0</v>
+        <v>2.0</v>
       </c>
       <c r="L27" t="n" s="0">
-        <v>-1.0</v>
+        <v>1.0</v>
       </c>
       <c r="M27" t="n" s="0">
-        <v>-1.0</v>
+        <v>3.0</v>
       </c>
       <c r="N27" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="O27" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="P27" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="Q27" t="n" s="0">
-        <v>-1.0</v>
+        <v>7.0</v>
       </c>
     </row>
     <row r="28">
@@ -1492,34 +1492,34 @@
         <v>0.0</v>
       </c>
       <c r="H28" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="I28" t="n" s="0">
         <v>-1.0</v>
       </c>
       <c r="J28" t="n" s="0">
-        <v>-1.0</v>
+        <v>105.0</v>
       </c>
       <c r="K28" t="n" s="0">
-        <v>-1.0</v>
+        <v>57.0</v>
       </c>
       <c r="L28" t="n" s="0">
-        <v>-1.0</v>
+        <v>15.0</v>
       </c>
       <c r="M28" t="n" s="0">
-        <v>-1.0</v>
+        <v>72.0</v>
       </c>
       <c r="N28" t="n" s="0">
-        <v>-1.0</v>
+        <v>3.0</v>
       </c>
       <c r="O28" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="P28" t="n" s="0">
-        <v>-1.0</v>
+        <v>6.0</v>
       </c>
       <c r="Q28" t="n" s="0">
-        <v>-1.0</v>
+        <v>80.0</v>
       </c>
     </row>
     <row r="29">
@@ -1539,34 +1539,34 @@
         <v>0.0</v>
       </c>
       <c r="H29" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="I29" t="n" s="0">
         <v>-1.0</v>
       </c>
       <c r="J29" t="n" s="0">
-        <v>-1.0</v>
+        <v>1.0</v>
       </c>
       <c r="K29" t="n" s="0">
-        <v>-1.0</v>
+        <v>11.0</v>
       </c>
       <c r="L29" t="n" s="0">
-        <v>-1.0</v>
+        <v>2.0</v>
       </c>
       <c r="M29" t="n" s="0">
-        <v>-1.0</v>
+        <v>13.0</v>
       </c>
       <c r="N29" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="O29" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="P29" t="n" s="0">
-        <v>-1.0</v>
+        <v>2.0</v>
       </c>
       <c r="Q29" t="n" s="0">
-        <v>-1.0</v>
+        <v>19.0</v>
       </c>
     </row>
     <row r="30">
@@ -1586,34 +1586,34 @@
         <v>0.0</v>
       </c>
       <c r="H30" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="I30" t="n" s="0">
         <v>-1.0</v>
       </c>
       <c r="J30" t="n" s="0">
-        <v>-1.0</v>
+        <v>28.0</v>
       </c>
       <c r="K30" t="n" s="0">
-        <v>-1.0</v>
+        <v>17.0</v>
       </c>
       <c r="L30" t="n" s="0">
-        <v>-1.0</v>
+        <v>8.0</v>
       </c>
       <c r="M30" t="n" s="0">
-        <v>-1.0</v>
+        <v>25.0</v>
       </c>
       <c r="N30" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="O30" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="P30" t="n" s="0">
-        <v>-1.0</v>
+        <v>3.0</v>
       </c>
       <c r="Q30" t="n" s="0">
-        <v>-1.0</v>
+        <v>70.0</v>
       </c>
     </row>
     <row r="31">
@@ -1633,34 +1633,34 @@
         <v>0.0</v>
       </c>
       <c r="H31" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="I31" t="n" s="0">
         <v>-1.0</v>
       </c>
       <c r="J31" t="n" s="0">
-        <v>-1.0</v>
+        <v>3.0</v>
       </c>
       <c r="K31" t="n" s="0">
-        <v>-1.0</v>
+        <v>3.0</v>
       </c>
       <c r="L31" t="n" s="0">
-        <v>-1.0</v>
+        <v>3.0</v>
       </c>
       <c r="M31" t="n" s="0">
-        <v>-1.0</v>
+        <v>6.0</v>
       </c>
       <c r="N31" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="O31" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="P31" t="n" s="0">
-        <v>-1.0</v>
+        <v>1.0</v>
       </c>
       <c r="Q31" t="n" s="0">
-        <v>-1.0</v>
+        <v>14.0</v>
       </c>
     </row>
     <row r="32">
@@ -1680,34 +1680,34 @@
         <v>0.0</v>
       </c>
       <c r="H32" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="I32" t="n" s="0">
         <v>-1.0</v>
       </c>
       <c r="J32" t="n" s="0">
-        <v>-1.0</v>
+        <v>28.0</v>
       </c>
       <c r="K32" t="n" s="0">
-        <v>-1.0</v>
+        <v>19.0</v>
       </c>
       <c r="L32" t="n" s="0">
-        <v>-1.0</v>
+        <v>8.0</v>
       </c>
       <c r="M32" t="n" s="0">
-        <v>-1.0</v>
+        <v>27.0</v>
       </c>
       <c r="N32" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="O32" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="P32" t="n" s="0">
-        <v>-1.0</v>
+        <v>2.0</v>
       </c>
       <c r="Q32" t="n" s="0">
-        <v>-1.0</v>
+        <v>56.0</v>
       </c>
     </row>
     <row r="33">
@@ -1727,34 +1727,34 @@
         <v>0.0</v>
       </c>
       <c r="H33" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="I33" t="n" s="0">
         <v>-1.0</v>
       </c>
       <c r="J33" t="n" s="0">
-        <v>-1.0</v>
+        <v>120.0</v>
       </c>
       <c r="K33" t="n" s="0">
-        <v>-1.0</v>
+        <v>42.0</v>
       </c>
       <c r="L33" t="n" s="0">
-        <v>-1.0</v>
+        <v>16.0</v>
       </c>
       <c r="M33" t="n" s="0">
-        <v>-1.0</v>
+        <v>58.0</v>
       </c>
       <c r="N33" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="O33" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="P33" t="n" s="0">
-        <v>-1.0</v>
+        <v>2.0</v>
       </c>
       <c r="Q33" t="n" s="0">
-        <v>-1.0</v>
+        <v>134.0</v>
       </c>
     </row>
     <row r="34">
@@ -1774,34 +1774,34 @@
         <v>0.0</v>
       </c>
       <c r="H34" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="I34" t="n" s="0">
         <v>-1.0</v>
       </c>
       <c r="J34" t="n" s="0">
-        <v>-1.0</v>
+        <v>3.0</v>
       </c>
       <c r="K34" t="n" s="0">
-        <v>-1.0</v>
+        <v>17.0</v>
       </c>
       <c r="L34" t="n" s="0">
-        <v>-1.0</v>
+        <v>3.0</v>
       </c>
       <c r="M34" t="n" s="0">
-        <v>-1.0</v>
+        <v>20.0</v>
       </c>
       <c r="N34" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="O34" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="P34" t="n" s="0">
-        <v>-1.0</v>
+        <v>4.0</v>
       </c>
       <c r="Q34" t="n" s="0">
-        <v>-1.0</v>
+        <v>47.0</v>
       </c>
     </row>
     <row r="35">
@@ -1821,34 +1821,34 @@
         <v>0.0</v>
       </c>
       <c r="H35" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="I35" t="n" s="0">
         <v>-1.0</v>
       </c>
       <c r="J35" t="n" s="0">
-        <v>-1.0</v>
+        <v>28.0</v>
       </c>
       <c r="K35" t="n" s="0">
-        <v>-1.0</v>
+        <v>31.0</v>
       </c>
       <c r="L35" t="n" s="0">
-        <v>-1.0</v>
+        <v>8.0</v>
       </c>
       <c r="M35" t="n" s="0">
-        <v>-1.0</v>
+        <v>39.0</v>
       </c>
       <c r="N35" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="O35" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="P35" t="n" s="0">
-        <v>-1.0</v>
+        <v>4.0</v>
       </c>
       <c r="Q35" t="n" s="0">
-        <v>-1.0</v>
+        <v>77.0</v>
       </c>
     </row>
     <row r="36">
@@ -1868,34 +1868,34 @@
         <v>0.0</v>
       </c>
       <c r="H36" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="I36" t="n" s="0">
         <v>-1.0</v>
       </c>
       <c r="J36" t="n" s="0">
-        <v>-1.0</v>
+        <v>6.0</v>
       </c>
       <c r="K36" t="n" s="0">
-        <v>-1.0</v>
+        <v>16.0</v>
       </c>
       <c r="L36" t="n" s="0">
-        <v>-1.0</v>
+        <v>4.0</v>
       </c>
       <c r="M36" t="n" s="0">
-        <v>-1.0</v>
+        <v>20.0</v>
       </c>
       <c r="N36" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="O36" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="P36" t="n" s="0">
-        <v>-1.0</v>
+        <v>1.0</v>
       </c>
       <c r="Q36" t="n" s="0">
-        <v>-1.0</v>
+        <v>37.0</v>
       </c>
     </row>
     <row r="37">
@@ -1915,34 +1915,34 @@
         <v>0.0</v>
       </c>
       <c r="H37" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="I37" t="n" s="0">
         <v>-1.0</v>
       </c>
       <c r="J37" t="n" s="0">
-        <v>-1.0</v>
+        <v>6.0</v>
       </c>
       <c r="K37" t="n" s="0">
-        <v>-1.0</v>
+        <v>19.0</v>
       </c>
       <c r="L37" t="n" s="0">
-        <v>-1.0</v>
+        <v>4.0</v>
       </c>
       <c r="M37" t="n" s="0">
-        <v>-1.0</v>
+        <v>23.0</v>
       </c>
       <c r="N37" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="O37" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="P37" t="n" s="0">
-        <v>-1.0</v>
+        <v>2.0</v>
       </c>
       <c r="Q37" t="n" s="0">
-        <v>-1.0</v>
+        <v>28.0</v>
       </c>
     </row>
     <row r="38">
@@ -1962,34 +1962,34 @@
         <v>0.0</v>
       </c>
       <c r="H38" t="n" s="0">
-        <v>-1.0</v>
+        <v>1.0</v>
       </c>
       <c r="I38" t="n" s="0">
         <v>-1.0</v>
       </c>
       <c r="J38" t="n" s="0">
-        <v>-1.0</v>
+        <v>28.0</v>
       </c>
       <c r="K38" t="n" s="0">
-        <v>-1.0</v>
+        <v>6.0</v>
       </c>
       <c r="L38" t="n" s="0">
-        <v>-1.0</v>
+        <v>8.0</v>
       </c>
       <c r="M38" t="n" s="0">
-        <v>-1.0</v>
+        <v>14.0</v>
       </c>
       <c r="N38" t="n" s="0">
-        <v>-1.0</v>
+        <v>1.0</v>
       </c>
       <c r="O38" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="P38" t="n" s="0">
-        <v>-1.0</v>
+        <v>2.0</v>
       </c>
       <c r="Q38" t="n" s="0">
-        <v>-1.0</v>
+        <v>31.0</v>
       </c>
     </row>
     <row r="39">
@@ -2009,34 +2009,34 @@
         <v>0.0</v>
       </c>
       <c r="H39" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="I39" t="n" s="0">
         <v>-1.0</v>
       </c>
       <c r="J39" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="K39" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="L39" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="M39" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="N39" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="O39" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="P39" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="Q39" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
     </row>
     <row r="40">
@@ -2056,34 +2056,34 @@
         <v>0.0</v>
       </c>
       <c r="H40" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="I40" t="n" s="0">
         <v>-1.0</v>
       </c>
       <c r="J40" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="K40" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="L40" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="M40" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="N40" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="O40" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="P40" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="Q40" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
     </row>
     <row r="41">
@@ -2103,34 +2103,34 @@
         <v>0.0</v>
       </c>
       <c r="H41" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="I41" t="n" s="0">
         <v>-1.0</v>
       </c>
       <c r="J41" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="K41" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="L41" t="n" s="0">
-        <v>-1.0</v>
+        <v>1.0</v>
       </c>
       <c r="M41" t="n" s="0">
-        <v>-1.0</v>
+        <v>1.0</v>
       </c>
       <c r="N41" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="O41" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="P41" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="Q41" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
     </row>
     <row r="42">
@@ -2150,34 +2150,34 @@
         <v>0.0</v>
       </c>
       <c r="H42" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="I42" t="n" s="0">
         <v>-1.0</v>
       </c>
       <c r="J42" t="n" s="0">
-        <v>-1.0</v>
+        <v>1.0</v>
       </c>
       <c r="K42" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="L42" t="n" s="0">
-        <v>-1.0</v>
+        <v>2.0</v>
       </c>
       <c r="M42" t="n" s="0">
-        <v>-1.0</v>
+        <v>2.0</v>
       </c>
       <c r="N42" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="O42" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="P42" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="Q42" t="n" s="0">
-        <v>-1.0</v>
+        <v>4.0</v>
       </c>
     </row>
     <row r="43">
@@ -2197,34 +2197,34 @@
         <v>0.0</v>
       </c>
       <c r="H43" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="I43" t="n" s="0">
         <v>-1.0</v>
       </c>
       <c r="J43" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="K43" t="n" s="0">
-        <v>-1.0</v>
+        <v>2.0</v>
       </c>
       <c r="L43" t="n" s="0">
-        <v>-1.0</v>
+        <v>1.0</v>
       </c>
       <c r="M43" t="n" s="0">
-        <v>-1.0</v>
+        <v>3.0</v>
       </c>
       <c r="N43" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="O43" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="P43" t="n" s="0">
-        <v>-1.0</v>
+        <v>1.0</v>
       </c>
       <c r="Q43" t="n" s="0">
-        <v>-1.0</v>
+        <v>13.0</v>
       </c>
     </row>
     <row r="44">
@@ -2244,34 +2244,34 @@
         <v>0.0</v>
       </c>
       <c r="H44" t="n" s="0">
-        <v>-1.0</v>
+        <v>1.0</v>
       </c>
       <c r="I44" t="n" s="0">
         <v>-1.0</v>
       </c>
       <c r="J44" t="n" s="0">
-        <v>-1.0</v>
+        <v>276.0</v>
       </c>
       <c r="K44" t="n" s="0">
-        <v>-1.0</v>
+        <v>14.0</v>
       </c>
       <c r="L44" t="n" s="0">
-        <v>-1.0</v>
+        <v>24.0</v>
       </c>
       <c r="M44" t="n" s="0">
-        <v>-1.0</v>
+        <v>38.0</v>
       </c>
       <c r="N44" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="O44" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="P44" t="n" s="0">
-        <v>-1.0</v>
+        <v>2.0</v>
       </c>
       <c r="Q44" t="n" s="0">
-        <v>-1.0</v>
+        <v>146.0</v>
       </c>
     </row>
     <row r="45">
@@ -2291,34 +2291,34 @@
         <v>0.0</v>
       </c>
       <c r="H45" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="I45" t="n" s="0">
         <v>-1.0</v>
       </c>
       <c r="J45" t="n" s="0">
-        <v>-1.0</v>
+        <v>406.0</v>
       </c>
       <c r="K45" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="L45" t="n" s="0">
-        <v>-1.0</v>
+        <v>29.0</v>
       </c>
       <c r="M45" t="n" s="0">
-        <v>-1.0</v>
+        <v>29.0</v>
       </c>
       <c r="N45" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="O45" t="n" s="0">
-        <v>-1.0</v>
+        <v>2.0</v>
       </c>
       <c r="P45" t="n" s="0">
-        <v>-1.0</v>
+        <v>1.0</v>
       </c>
       <c r="Q45" t="n" s="0">
-        <v>-1.0</v>
+        <v>83.0</v>
       </c>
     </row>
     <row r="46">
@@ -2338,34 +2338,34 @@
         <v>0.0</v>
       </c>
       <c r="H46" t="n" s="0">
-        <v>-1.0</v>
+        <v>2.0</v>
       </c>
       <c r="I46" t="n" s="0">
         <v>-1.0</v>
       </c>
       <c r="J46" t="n" s="0">
-        <v>-1.0</v>
+        <v>6.0</v>
       </c>
       <c r="K46" t="n" s="0">
-        <v>-1.0</v>
+        <v>30.0</v>
       </c>
       <c r="L46" t="n" s="0">
-        <v>-1.0</v>
+        <v>4.0</v>
       </c>
       <c r="M46" t="n" s="0">
-        <v>-1.0</v>
+        <v>34.0</v>
       </c>
       <c r="N46" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="O46" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="P46" t="n" s="0">
-        <v>-1.0</v>
+        <v>4.0</v>
       </c>
       <c r="Q46" t="n" s="0">
-        <v>-1.0</v>
+        <v>74.0</v>
       </c>
     </row>
     <row r="47">
@@ -2385,34 +2385,34 @@
         <v>0.0</v>
       </c>
       <c r="H47" t="n" s="0">
-        <v>-1.0</v>
+        <v>2.0</v>
       </c>
       <c r="I47" t="n" s="0">
         <v>-1.0</v>
       </c>
       <c r="J47" t="n" s="0">
-        <v>-1.0</v>
+        <v>3.0</v>
       </c>
       <c r="K47" t="n" s="0">
-        <v>-1.0</v>
+        <v>12.0</v>
       </c>
       <c r="L47" t="n" s="0">
-        <v>-1.0</v>
+        <v>3.0</v>
       </c>
       <c r="M47" t="n" s="0">
-        <v>-1.0</v>
+        <v>15.0</v>
       </c>
       <c r="N47" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="O47" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="P47" t="n" s="0">
-        <v>-1.0</v>
+        <v>3.0</v>
       </c>
       <c r="Q47" t="n" s="0">
-        <v>-1.0</v>
+        <v>45.0</v>
       </c>
     </row>
     <row r="48">
@@ -2432,34 +2432,34 @@
         <v>0.0</v>
       </c>
       <c r="H48" t="n" s="0">
-        <v>-1.0</v>
+        <v>1.0</v>
       </c>
       <c r="I48" t="n" s="0">
         <v>-1.0</v>
       </c>
       <c r="J48" t="n" s="0">
-        <v>-1.0</v>
+        <v>21.0</v>
       </c>
       <c r="K48" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="L48" t="n" s="0">
-        <v>-1.0</v>
+        <v>7.0</v>
       </c>
       <c r="M48" t="n" s="0">
-        <v>-1.0</v>
+        <v>7.0</v>
       </c>
       <c r="N48" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="O48" t="n" s="0">
-        <v>-1.0</v>
+        <v>2.0</v>
       </c>
       <c r="P48" t="n" s="0">
-        <v>-1.0</v>
+        <v>2.0</v>
       </c>
       <c r="Q48" t="n" s="0">
-        <v>-1.0</v>
+        <v>20.0</v>
       </c>
     </row>
     <row r="49">
@@ -2479,34 +2479,34 @@
         <v>0.0</v>
       </c>
       <c r="H49" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="I49" t="n" s="0">
         <v>-1.0</v>
       </c>
       <c r="J49" t="n" s="0">
-        <v>-1.0</v>
+        <v>1.0</v>
       </c>
       <c r="K49" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="L49" t="n" s="0">
-        <v>-1.0</v>
+        <v>2.0</v>
       </c>
       <c r="M49" t="n" s="0">
-        <v>-1.0</v>
+        <v>2.0</v>
       </c>
       <c r="N49" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="O49" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="P49" t="n" s="0">
-        <v>-1.0</v>
+        <v>2.0</v>
       </c>
       <c r="Q49" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
     </row>
     <row r="50">
@@ -2526,34 +2526,34 @@
         <v>0.0</v>
       </c>
       <c r="H50" t="n" s="0">
-        <v>-1.0</v>
+        <v>1.0</v>
       </c>
       <c r="I50" t="n" s="0">
         <v>-1.0</v>
       </c>
       <c r="J50" t="n" s="0">
-        <v>-1.0</v>
+        <v>10.0</v>
       </c>
       <c r="K50" t="n" s="0">
-        <v>-1.0</v>
+        <v>16.0</v>
       </c>
       <c r="L50" t="n" s="0">
-        <v>-1.0</v>
+        <v>5.0</v>
       </c>
       <c r="M50" t="n" s="0">
-        <v>-1.0</v>
+        <v>21.0</v>
       </c>
       <c r="N50" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="O50" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="P50" t="n" s="0">
-        <v>-1.0</v>
+        <v>3.0</v>
       </c>
       <c r="Q50" t="n" s="0">
-        <v>-1.0</v>
+        <v>47.0</v>
       </c>
     </row>
     <row r="51">
@@ -2573,34 +2573,34 @@
         <v>0.0</v>
       </c>
       <c r="H51" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="I51" t="n" s="0">
         <v>-1.0</v>
       </c>
       <c r="J51" t="n" s="0">
-        <v>-1.0</v>
+        <v>861.0</v>
       </c>
       <c r="K51" t="n" s="0">
-        <v>-1.0</v>
+        <v>205.0</v>
       </c>
       <c r="L51" t="n" s="0">
-        <v>-1.0</v>
+        <v>42.0</v>
       </c>
       <c r="M51" t="n" s="0">
-        <v>-1.0</v>
+        <v>247.0</v>
       </c>
       <c r="N51" t="n" s="0">
-        <v>-1.0</v>
+        <v>2.0</v>
       </c>
       <c r="O51" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="P51" t="n" s="0">
-        <v>-1.0</v>
+        <v>4.0</v>
       </c>
       <c r="Q51" t="n" s="0">
-        <v>-1.0</v>
+        <v>606.0</v>
       </c>
     </row>
     <row r="52">
@@ -2620,34 +2620,34 @@
         <v>0.0</v>
       </c>
       <c r="H52" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="I52" t="n" s="0">
         <v>-1.0</v>
       </c>
       <c r="J52" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="K52" t="n" s="0">
-        <v>-1.0</v>
+        <v>2.0</v>
       </c>
       <c r="L52" t="n" s="0">
-        <v>-1.0</v>
+        <v>1.0</v>
       </c>
       <c r="M52" t="n" s="0">
-        <v>-1.0</v>
+        <v>3.0</v>
       </c>
       <c r="N52" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="O52" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="P52" t="n" s="0">
-        <v>-1.0</v>
+        <v>0.0</v>
       </c>
       <c r="Q52" t="n" s="0">
-        <v>-1.0</v>
+        <v>7.0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>